<commit_message>
added excelfile for register map for project
</commit_message>
<xml_diff>
--- a/ECE2031_ADC_Peripheral_Register_Map_Lab06G5.xlsx
+++ b/ECE2031_ADC_Peripheral_Register_Map_Lab06G5.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://gtvault-my.sharepoint.com/personal/kly36_gatech_edu/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kevly\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="8_{2CDA5EC3-09A3-47FA-AEBB-0E11C7B06680}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BE55D582-0FD9-42A1-976F-FACBF3FBCB41}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92CB85A7-379E-4A3C-AFAB-E97B42E76654}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2508" yWindow="5136" windowWidth="17280" windowHeight="9960" xr2:uid="{D04FC250-84EE-4908-9CFF-BD242F277824}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{D04FC250-84EE-4908-9CFF-BD242F277824}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,16 +36,142 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1" uniqueCount="1">
-  <si>
-    <t>test</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="43">
+  <si>
+    <t>Register</t>
+  </si>
+  <si>
+    <t>Register Name</t>
+  </si>
+  <si>
+    <t>B15</t>
+  </si>
+  <si>
+    <t>B14</t>
+  </si>
+  <si>
+    <t>B13</t>
+  </si>
+  <si>
+    <t>B12</t>
+  </si>
+  <si>
+    <t>B11</t>
+  </si>
+  <si>
+    <t>B10</t>
+  </si>
+  <si>
+    <t>B9</t>
+  </si>
+  <si>
+    <t>B8</t>
+  </si>
+  <si>
+    <t>B7</t>
+  </si>
+  <si>
+    <t>B6</t>
+  </si>
+  <si>
+    <t>B5</t>
+  </si>
+  <si>
+    <t>B4</t>
+  </si>
+  <si>
+    <t>B3</t>
+  </si>
+  <si>
+    <t>B2</t>
+  </si>
+  <si>
+    <t>B1</t>
+  </si>
+  <si>
+    <t>B0</t>
+  </si>
+  <si>
+    <t>0xC0</t>
+  </si>
+  <si>
+    <t>ADC_CTRL</t>
+  </si>
+  <si>
+    <t>Channel</t>
+  </si>
+  <si>
+    <t>clear_ready</t>
+  </si>
+  <si>
+    <t>start</t>
+  </si>
+  <si>
+    <t>0xC1</t>
+  </si>
+  <si>
+    <t>ADC_STATUS</t>
+  </si>
+  <si>
+    <t>busy</t>
+  </si>
+  <si>
+    <t>ready</t>
+  </si>
+  <si>
+    <t>0xC2</t>
+  </si>
+  <si>
+    <t>ADC_DATA</t>
+  </si>
+  <si>
+    <t>0xC3</t>
+  </si>
+  <si>
+    <t>Chan_Info</t>
+  </si>
+  <si>
+    <t>0xC4</t>
+  </si>
+  <si>
+    <t>0xC5</t>
+  </si>
+  <si>
+    <t>0xC6</t>
+  </si>
+  <si>
+    <t>0xC7</t>
+  </si>
+  <si>
+    <t>0xC8</t>
+  </si>
+  <si>
+    <t>0xC9</t>
+  </si>
+  <si>
+    <t>0xCA</t>
+  </si>
+  <si>
+    <t>0xCB</t>
+  </si>
+  <si>
+    <t>0xCC</t>
+  </si>
+  <si>
+    <t>0xCD</t>
+  </si>
+  <si>
+    <t>0xCE</t>
+  </si>
+  <si>
+    <t>0xCF</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -53,16 +179,36 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="1" tint="0.499984740745262"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -70,12 +216,31 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -410,12 +575,251 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7BE48722-12FD-4C51-A763-702FD7C97D36}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:R17"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="12.77734375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="10.33203125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
         <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
+      <c r="I2" s="2"/>
+      <c r="J2" s="2"/>
+      <c r="K2" s="2"/>
+      <c r="L2" s="2"/>
+      <c r="M2" s="2"/>
+      <c r="N2" t="s">
+        <v>20</v>
+      </c>
+      <c r="O2" t="s">
+        <v>20</v>
+      </c>
+      <c r="P2" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>21</v>
+      </c>
+      <c r="R2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+      <c r="I3" s="2"/>
+      <c r="J3" s="2"/>
+      <c r="K3" s="2"/>
+      <c r="L3" s="2"/>
+      <c r="M3" s="2"/>
+      <c r="N3" s="2"/>
+      <c r="O3" s="2"/>
+      <c r="P3" s="2"/>
+      <c r="Q3" t="s">
+        <v>25</v>
+      </c>
+      <c r="R3" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C4">
+        <v>0</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4">
+        <v>0</v>
+      </c>
+      <c r="G4" s="2"/>
+      <c r="H4" s="2"/>
+      <c r="I4" s="2"/>
+      <c r="J4" s="2"/>
+      <c r="K4" s="2"/>
+      <c r="L4" s="2"/>
+      <c r="M4" s="2"/>
+      <c r="N4" s="2"/>
+      <c r="O4" s="2"/>
+      <c r="P4" s="2"/>
+      <c r="Q4" s="2"/>
+      <c r="R4" s="2"/>
+    </row>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>29</v>
+      </c>
+      <c r="B5" t="s">
+        <v>30</v>
+      </c>
+      <c r="C5" s="2"/>
+      <c r="D5" s="2"/>
+      <c r="E5" s="2"/>
+      <c r="F5" s="2"/>
+      <c r="G5" s="2"/>
+      <c r="H5" s="2"/>
+      <c r="I5" s="2"/>
+      <c r="J5" s="2"/>
+      <c r="K5" s="2"/>
+      <c r="L5" s="2"/>
+      <c r="M5" s="2"/>
+      <c r="N5" s="2"/>
+      <c r="O5" s="2"/>
+      <c r="P5" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>20</v>
+      </c>
+      <c r="R5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="7" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="8" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="10" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="11" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="12" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="13" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="14" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="15" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="16" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>42</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Changed channel bits to match throughout Register Map
</commit_message>
<xml_diff>
--- a/ECE2031_ADC_Peripheral_Register_Map_Lab06G5.xlsx
+++ b/ECE2031_ADC_Peripheral_Register_Map_Lab06G5.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kevly\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kevly\Downloads\ece2031stuff\ece2031-project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92CB85A7-379E-4A3C-AFAB-E97B42E76654}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7C40050-3E94-4ED1-AAFC-DD8CF46D5FFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{D04FC250-84EE-4908-9CFF-BD242F277824}"/>
   </bookViews>
@@ -750,17 +750,17 @@
       <c r="K5" s="2"/>
       <c r="L5" s="2"/>
       <c r="M5" s="2"/>
-      <c r="N5" s="2"/>
-      <c r="O5" s="2"/>
+      <c r="N5" t="s">
+        <v>20</v>
+      </c>
+      <c r="O5" t="s">
+        <v>20</v>
+      </c>
       <c r="P5" t="s">
         <v>20</v>
       </c>
-      <c r="Q5" t="s">
-        <v>20</v>
-      </c>
-      <c r="R5" t="s">
-        <v>20</v>
-      </c>
+      <c r="Q5" s="2"/>
+      <c r="R5" s="2"/>
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A6" t="s">

</xml_diff>